<commit_message>
Fichas Excel: cobertura de basura con una casilla por clase para marcar con X
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6fB2a98KHteXa37uYKffB
</commit_message>
<xml_diff>
--- a/resultados/campo/fichas_excel/Ficha_P01.xlsx
+++ b/resultados/campo/fichas_excel/Ficha_P01.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -662,40 +662,81 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Basura que tapa el agua de frente (hasta ~50 m)</t>
+          <t>Basura que tapa el agua: ninguna</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>☐</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Olor</t>
+          <t>Basura que tapa el agua: poca (menos de 1 de cada 10 partes)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>☐</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Si «otro», ¿cuál? (olor)</t>
+          <t>Basura que tapa el agua: bastante (1 a 5 de 10)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>☐</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>3. Fotos de la nº</t>
+          <t>Basura que tapa el agua: mucha (más de 5 de 10)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>☐</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Fotos hasta la nº</t>
+          <t>Olor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Si «otro», ¿cuál? (olor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>3. Fotos de la nº</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Fotos hasta la nº</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -705,7 +746,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <dataValidations count="14">
+  <dataValidations count="17">
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3"</formula1>
     </dataValidation>
@@ -743,9 +784,18 @@
       <formula1>"☐,☒"</formula1>
     </dataValidation>
     <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ninguna,poca (menos de 1 de 10),bastante (1 a 5 de 10),mucha (más de 5 de 10)"</formula1>
+      <formula1>"☐,☒"</formula1>
     </dataValidation>
     <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"☐,☒"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"☐,☒"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"☐,☒"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ninguno,a cloaca,a químico o combustible,otro"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>